<commit_message>
PLC Logic & Testing Doc
- More Testing was done this evening (10/7)
</commit_message>
<xml_diff>
--- a/Testing Documentation/10-6-ValveTestRateOfChangeActuation.xlsx
+++ b/Testing Documentation/10-6-ValveTestRateOfChangeActuation.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96325486694b1ce6/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96325486694b1ce6/Documents/GitHub/TMEIC-DI-Water-Cooling-Skid-Repo/Testing Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F659A72-B4FD-4EF3-8D4F-B6780C30CDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{2F659A72-B4FD-4EF3-8D4F-B6780C30CDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DBF58DD-1ED1-46C0-A548-1F84E2E1E395}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{10D479EA-35C7-4C0B-9B4E-B3672E68B92B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1717,7 +1717,7 @@
         <v>0.50549500000000003</v>
       </c>
       <c r="K2">
-        <f>I2-J2</f>
+        <f t="shared" ref="K2:K12" si="0">I2-J2</f>
         <v>12.813185000000001</v>
       </c>
       <c r="L2">
@@ -1744,11 +1744,11 @@
         <v>27.648350000000001</v>
       </c>
       <c r="K3">
-        <f>I3-J3</f>
+        <f t="shared" si="0"/>
         <v>13.406599999999997</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3:L12" si="0">K3/H3</f>
+        <f t="shared" ref="L3:L12" si="1">K3/H3</f>
         <v>3.6932782369145971</v>
       </c>
       <c r="M3">
@@ -1771,11 +1771,11 @@
         <v>41.054949999999998</v>
       </c>
       <c r="K4">
-        <f>I4-J4</f>
+        <f t="shared" si="0"/>
         <v>14.142850000000003</v>
       </c>
       <c r="L4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.553479899497491</v>
       </c>
       <c r="M4">
@@ -1798,11 +1798,11 @@
         <v>55.241759999999999</v>
       </c>
       <c r="K5">
-        <f>I5-J5</f>
+        <f t="shared" si="0"/>
         <v>13.362629999999996</v>
       </c>
       <c r="L5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.7211445279866235</v>
       </c>
       <c r="M5">
@@ -1825,11 +1825,11 @@
         <v>68.692310000000006</v>
       </c>
       <c r="K6">
-        <f>I6-J6</f>
+        <f t="shared" si="0"/>
         <v>13.516479999999987</v>
       </c>
       <c r="L6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.6403124158362394</v>
       </c>
       <c r="M6">
@@ -1852,11 +1852,11 @@
         <v>82.252750000000006</v>
       </c>
       <c r="K7">
-        <f>I7-J7</f>
+        <f t="shared" si="0"/>
         <v>7.6922999999999888</v>
       </c>
       <c r="L7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.1029850746268623</v>
       </c>
       <c r="M7">
@@ -1879,11 +1879,11 @@
         <v>6.5934099999999995E-2</v>
       </c>
       <c r="K8">
-        <f>I8-J8</f>
+        <f t="shared" si="0"/>
         <v>89.879115899999988</v>
       </c>
       <c r="L8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.7813126875199474</v>
       </c>
       <c r="M8">
@@ -1906,11 +1906,11 @@
         <v>2.1978000000000001E-2</v>
       </c>
       <c r="K9">
-        <f>I9-J9</f>
+        <f t="shared" si="0"/>
         <v>22.461541999999998</v>
       </c>
       <c r="L9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.8988963721576142</v>
       </c>
       <c r="M9">
@@ -1933,11 +1933,11 @@
         <v>22.527470000000001</v>
       </c>
       <c r="K10">
-        <f>I10-J10</f>
+        <f t="shared" si="0"/>
         <v>22.516489999999997</v>
       </c>
       <c r="L10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.1930148975791397</v>
       </c>
       <c r="M10">
@@ -1960,11 +1960,11 @@
         <v>45.087910000000001</v>
       </c>
       <c r="K11">
-        <f>I11-J11</f>
+        <f t="shared" si="0"/>
         <v>22.307690000000001</v>
       </c>
       <c r="L11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.2002805498022919</v>
       </c>
       <c r="M11">
@@ -1987,11 +1987,11 @@
         <v>67.43956</v>
       </c>
       <c r="K12">
-        <f>I12-J12</f>
+        <f t="shared" si="0"/>
         <v>22.395600000000002</v>
       </c>
       <c r="L12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.1010071415491574</v>
       </c>
       <c r="M12">
@@ -2013,52 +2013,60 @@
     <row r="16" spans="6:14" x14ac:dyDescent="0.3">
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="L20">
+        <f>_xlfn.VAR.P(L2:L12)</f>
+        <v>0.19779628084327761</v>
+      </c>
+    </row>
+    <row r="21" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="L21">
+        <f>_xlfn.STDEV.P(L2:L12)</f>
+        <v>0.44474293793524999</v>
+      </c>
+    </row>
+    <row r="22" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F30" s="1"/>
     </row>
-    <row r="31" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F31" s="1"/>
     </row>
-    <row r="32" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="6:6" x14ac:dyDescent="0.3">

</xml_diff>